<commit_message>
Initial state: CMMS project before improvements - Code analysis and assessment complete
</commit_message>
<xml_diff>
--- a/data/gebze/rca_analysis.xlsx
+++ b/data/gebze/rca_analysis.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -874,6 +874,174 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:28</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GDM2</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Batarya Hücreleri</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>servis_disi</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:28</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>GDM2</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Batarya Hücreleri</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>servis_disi</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:29</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>GDM2</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Batarya Hücreleri</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>servis_disi</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:30</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>GDM3</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pantograf</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Pantograf Kollektör Kafası</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>servis_disi</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:30</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>GDM1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Batarya Hücreleri</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>servis_disi</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:30</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>GDM7</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Lubrication_System</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Yağlama Kontrol ünitesi</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>servis_disi</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>